<commit_message>
Update berita 2026-08-05 05:19 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-02.xlsx
+++ b/data/berita_2026-08-02.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$H$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$H$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -895,33 +895,33 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Lifestyle</t>
+          <t>Tekno</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>20 ide hadiah lomba 17 Agustus 2026 yang murah, bermanfaat, dan menarik</t>
+          <t>10 cara mengurangi screen time agar mata tetap sehat dan tidur nyenyak</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Sun, 02 Aug 2026 11:09:39 +0700</t>
+          <t>Sun, 02 Aug 2026 10:13:01 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Menjelang peringatan HUT ke-81 Kemerdekaan Republik Indonesia pada 17 Agustus 2026, berbagai lingkungan mulai ...</t>
+          <t>Penggunaan ponsel, tablet, dan komputer telah menjadi bagian dari kehidupan sehari-hari. Mulai dari bekerja, belajar, ...</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676419/20-ide-hadiah-lomba-17-agustus-2026-yang-murah-bermanfaat-dan-menarik</t>
+          <t>https://www.antaranews.com/berita/5676376/10-cara-mengurangi-screen-time-agar-mata-tetap-sehat-dan-tidur-nyenyak</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2025/08/17/pesta-rakyat-hut-ri-di-monas-2602245.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/09/CDAD3117-892E-4E7F-AF44-CF43EED7F052.jpeg</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -938,28 +938,28 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10 cara mengurangi screen time agar mata tetap sehat dan tidur nyenyak</t>
+          <t>Cara tepat restart paksa iPhone yang error agar kembali normal</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Sun, 02 Aug 2026 10:13:01 +0700</t>
+          <t>Sun, 02 Aug 2026 10:09:15 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Penggunaan ponsel, tablet, dan komputer telah menjadi bagian dari kehidupan sehari-hari. Mulai dari bekerja, belajar, ...</t>
+          <t>iPhone yang tiba-tiba error, layar tidak merespons sentuhan, atau berhenti di logo Apple menjadi masalah yang cukup ...</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676376/10-cara-mengurangi-screen-time-agar-mata-tetap-sehat-dan-tidur-nyenyak</t>
+          <t>https://www.antaranews.com/berita/5676373/cara-tepat-restart-paksa-iphone-yang-error-agar-kembali-normal</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/09/CDAD3117-892E-4E7F-AF44-CF43EED7F052.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/13/InShot_20260513_153025843.jpg</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -968,46 +968,8 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Tekno</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Cara tepat restart paksa iPhone yang error agar kembali normal</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Sun, 02 Aug 2026 10:09:15 +0700</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>iPhone yang tiba-tiba error, layar tidak merespons sentuhan, atau berhenti di logo Apple menjadi masalah yang cukup ...</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5676373/cara-tepat-restart-paksa-iphone-yang-error-agar-kembali-normal</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/13/InShot_20260513_153025843.jpg</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Antara</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H15"/>
+  <autoFilter ref="A1:H14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-06 10:54 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-02.xlsx
+++ b/data/berita_2026-08-02.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,18 +419,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="60" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1091,8 +1091,337 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>15 Aplikasi Bikin Rekening Terkuras, Jutaan Warga RI Download</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Sun, 02 Aug 2026 21:00:30 +0700</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Waspadai 15 aplikasi berbahaya di Google Play Store yang dapat mencuri data pribadi dan informasi keuangan. Jutaan pengguna terancam oleh pinjol palsu.</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260802180530-37-755834/15-aplikasi-bikin-rekening-terkuras-jutaan-warga-ri-download</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2023/08/07/marak-penipu-wa-kuras-rekening-kominfo-bongkar-modusnya_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Ada Gerhana Matahari Total 12 Agustus, Di Sini Lokasinya</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Sun, 02 Aug 2026 20:30:59 +0700</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Gerhana Matahari Total akan terjadi pada 12 Agustus 2026.</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260802161959-37-755815/ada-gerhana-matahari-total-12-agustus-di-sini-lokasinya</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2024/04/09/proses-gerhana-matahari-di-as-reutersandrew-kelly_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Virus Berbahaya Serang Pengguna iPhone, Begini Cara Hentikannya</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Sun, 02 Aug 2026 17:45:28 +0700</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Serangan malware Darksword mencuri data dari ratusan juta iPhone. Pengguna disarankan untuk memperbarui iOS demi keamanan perangkat mereka.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260802152407-37-755812/virus-berbahaya-serang-pengguna-iphone-begini-cara-hentikannya</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/09/10/seseorang-memegang-iphone-17-selama-acara-apple-di-steve-jobs-theater-di-kampusnya-di-cupertino-california-as-9-september-2025-1757462206892_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Mammoth Purba Muncul Saat Sungai Danube Surut ke Level Terendah</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Sun, 02 Aug 2026 15:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Sisa-sisa yang diyakini sebagai mammoth purba ditemukan di Bulgaria utara setelah permukaan air Sungai Danube surut ke level terendah sepanjang sejarah.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260730075747-38-754942/mammoth-purba-muncul-saat-sungai-danube-surut-ke-level-terendah</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/07/30/europe-weatherbulgaria-mammoth-1785373054223_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>NASA Sudah Temukan Jejak Alien, di Sini Lokasinya</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Sun, 02 Aug 2026 14:45:00 +0700</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>NASA menemukan tanda kehidupan di Mars dari misi Viking 1976. Temuan ini memicu perdebatan ilmiah tentang kemungkinan adanya mikroorganisme di Planet Merah.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260802123951-37-755799/nasa-sudah-temukan-jejak-alien-di-sini-lokasinya</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/01/20/planet-mars-tidak-merah-1768864409444_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Transformasi Di Bawah Danantara, Telkomsel Tumbuh Sehat Semester I</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Sun, 02 Aug 2026 10:07:08 +0700</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Telkomsel mencatat pertumbuhan pendapatan 3,3% di Semester I 2026, didukung transformasi digital dan layanan berkualitas.</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260802100040-37-755783/transformasi-di-bawah-danantara-telkomsel-tumbuh-sehat-semester-i</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/02/dok-telkomsel-1785639992472_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>China Makin Seksi, Amerika Terpaksa Banting Harga</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Sun, 02 Aug 2026 09:15:00 +0700</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Persaingan AI antara AS dan China memanas. OpenAI memangkas harga model hingga 80% untuk tetap bersaing. Kebijakan ini diharapkan tidak mengganggu profit.</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260802085842-37-755776/china-makin-seksi-amerika-terpaksa-banting-harga</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2024/12/02/bendera-amerikas-serikat-as-dan-china-reutersflorence-loillustrationfile_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I14"/>
+  <autoFilter ref="A1:I21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-06 11:05 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-02.xlsx
+++ b/data/berita_2026-08-02.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,13 +419,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -1420,8 +1420,478 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>DJ Bravy Kagumi Cara Erika Carlina Rayakan Ultah Putranya di Panti Asuhan</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Sun, 02 Aug 2026 23:03:38 +0700</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Febryantino Nur Pratama</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Erika Carlina merayakan ulang tahun pertama putranya dengan anak-anak panti asuhan di Cibubur. DJ Bravy mengapresiasi ide sosial ini sebagai bentuk syukur.</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8601177/dj-bravy-kagumi-cara-erika-carlina-rayakan-ultah-putranya-di-panti-asuhan</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/01/erika-carlina-asyik-kulineran-tradisional-cicip-nasi-jamblang-hingga-gado-gado-1785596582403_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>DJ Bravy Sebut Hubungan dengan Erika Carlina Masih Saling Dukung</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Sun, 02 Aug 2026 22:02:39 +0700</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Febryantino Nur Pratama</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>DJ Bravy mengungkapkan hubungan baik dengan Erika Carlina setelah putus. Mereka kini bersahabat dan saling mendukung, meski tak berencana balikan.</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8601166/dj-bravy-sebut-hubungan-dengan-erika-carlina-masih-saling-dukung</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/11/11/momen-erika-carlina-dan-dj-bravy-makan-unagi-viral-hingga-jajanan-kaki-lima-1762857981563_43.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Chelsea Olivia Puji Mukjizat Tuhan Saat Ayah Operasi Jantung-Bisa Lari Lagi</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Sun, 02 Aug 2026 21:01:58 +0700</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Mauludi Rismoyo</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Chelsea Olivia menceritakan perjalanan 2026 sejauh ini. Ia mengaku merasakan kebaikan Tuhan.</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8601116/chelsea-olivia-puji-mukjizat-tuhan-saat-ayah-operasi-jantung-bisa-lari-lagi</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/02/chelsea-olivia-1785664170001_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>DJ Bravy Takjub Lihat Perkembangan Anak Erika Carlina di Usia Setahun</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Sun, 02 Aug 2026 20:02:42 +0700</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Febryantino Nur Pratama</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Perayaan ulang tahun pertama Andrew, putra Erika Carlina, berlangsung hangat di panti asuhan. DJ Bravy, yang dekat dengan Andrew, mengungkapkan kebahagiaannya.</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8601041/dj-bravy-takjub-lihat-perkembangan-anak-erika-carlina-di-usia-setahun</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/10/30/erika-carlina-dan-anak-1761812694632_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Tyna Dwi Jayanti Jualan Bitterballen, Tetap Menawan Meski Berkeringat</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Sun, 02 Aug 2026 19:09:19 +0700</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Mauludi Rismoyo</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Ada kabar baru dari Tyna Dwi Jayanti. Mantan istri Kenang Mirdad itu kini berjualan makanan.</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8601003/tyna-dwi-jayanti-jualan-bitterballen-tetap-menawan-meski-berkeringat</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/02/tyna-dwi-jayanti-1785658935117_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Selvi Kitty Pamer Baby Bump</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Sun, 02 Aug 2026 18:08:44 +0700</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Mauludi Rismoyo</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Penyanyi Selvi Kitty memamerkan baby bump. Begini pesonanya.</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8600938/selvi-kitty-pamer-baby-bump</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/02/selvi-kitty-1785655013858_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Erika Carlina Pilih Tak Gelar Pesta Mewah Rayakan Ultah Anak</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Sun, 02 Aug 2026 18:07:06 +0700</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Febryantino Nur Pratama</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Erika Carlina merayakan ulang tahun pertama putranya dengan berbagi kebahagiaan di panti asuhan. Ia berharap Andrew tumbuh menjadi anak yang baik dan pintar.</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8601237/erika-carlina-pilih-tak-gelar-pesta-mewah-rayakan-ultah-anak</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/04/04/erika-carlina-1775263803410_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Tantangan Kreator Baru di Industri TikTok</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Sun, 02 Aug 2026 17:55:44 +0700</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>prih febriani</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Industri TikTok Live di Indonesia bertransformasi, fokus pada kualitas konten dan komunitas.</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/music/d-8601230/tantangan-kreator-baru-di-industri-tiktok</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/08/14/ilustrasi-media-sosial-1755140697647_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Forestra 2026 Siap Digelar 29 Agustus</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Sun, 02 Aug 2026 17:19:50 +0700</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>prih febriani</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Forestra 2026 hadir di Orchid Forest Cikole, Lembang-Bandung pada 29 Agustus. Nikmati kolaborasi musik lintas genre dalam suasana alam yang menakjubkan.</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/music/d-8601163/forestra-2026-siap-digelar-29-agustus</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/02/forestra-2026-1785663188735_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Rigen Rakelna Bongkar Kebiasaan Parah Istri</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Sun, 02 Aug 2026 17:07:24 +0700</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Febryantino Nur Pratama</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Rigen Rakelna berbagi cerita lucu tentang kebiasaan mandi istrinya, Indah. Meski jarang mandi, mereka saling mengingatkan tanpa masalah dalam rumah tangga.</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8600875/rigen-rakelna-bongkar-kebiasaan-parah-istri</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/30/romantis-rigen-rakelna-ajak-istri-makan-malam-di-restoran-1785407446615_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I21"/>
+  <autoFilter ref="A1:I31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>